<commit_message>
Hold Management Development Institute pages for QA revision
</commit_message>
<xml_diff>
--- a/data/college-content-master.xlsx
+++ b/data/college-content-master.xlsx
@@ -526,17 +526,17 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped - existing pages protected</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Already Exists</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Checked</t>
         </is>
       </c>
     </row>
@@ -588,17 +588,17 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped - existing pages protected</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Already Exists</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Checked</t>
         </is>
       </c>
     </row>
@@ -650,17 +650,17 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped - existing pages protected</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Already Exists</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Checked</t>
         </is>
       </c>
     </row>
@@ -712,17 +712,17 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped - existing pages protected</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Already Exists</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Checked</t>
         </is>
       </c>
     </row>
@@ -774,17 +774,17 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped - existing pages protected</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Already Exists</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Checked</t>
         </is>
       </c>
     </row>
@@ -836,17 +836,17 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped - existing pages protected</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Already Exists</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Checked</t>
         </is>
       </c>
     </row>
@@ -898,17 +898,17 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped - existing pages protected</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Already Exists</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Checked</t>
         </is>
       </c>
     </row>
@@ -960,17 +960,17 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped - existing pages protected</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Already Exists</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Checked</t>
         </is>
       </c>
     </row>
@@ -1007,27 +1007,27 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.mdi.ac.in</t>
+          <t>https://support.google.com/websearch</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Pending Audit</t>
+          <t>47</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Research Complete</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Failed</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked - QA &lt;= 70 or critical failure</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1901,27 +1901,27 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.nmims.edu/</t>
+          <t>https://www.nmims.edu</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>Pending Audit</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Research Complete</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Blocked - QA &lt;= 70 or critical failure</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">

</xml_diff>

<commit_message>
Hold Jamia Millia Islamia pages for QA revision
</commit_message>
<xml_diff>
--- a/data/college-content-master.xlsx
+++ b/data/college-content-master.xlsx
@@ -1007,7 +1007,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://support.google.com/websearch</t>
+          <t>https://www.mdi.ac.in</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -2066,17 +2066,17 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped - existing pages protected</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Already Exists</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Checked</t>
         </is>
       </c>
     </row>
@@ -2096,32 +2096,44 @@
           <t>28</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.jmi.ac.in</t>
+          <t>https://www.jmi.ac.in/</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Pending Audit</t>
+          <t>51</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Research Complete</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Failed</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked - QA &lt;= 70 or critical failure</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">

</xml_diff>

<commit_message>
Publish independently generated pages for Indian Institute of Management Visakhapatnam
</commit_message>
<xml_diff>
--- a/data/college-content-master.xlsx
+++ b/data/college-content-master.xlsx
@@ -2113,7 +2113,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.jmi.ac.in/</t>
+          <t>https://www.jmi.ac.in</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2160,30 +2160,34 @@
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.iimv.ac.in</t>
+          <t>https://www.iimv.ac.in/</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Pending Audit</t>
+          <t>93</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Research Complete</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Eligible - Auto Publish</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">

</xml_diff>

<commit_message>
Update quality and live status for Indian Institute of Management Visakhapatnam
</commit_message>
<xml_diff>
--- a/data/college-content-master.xlsx
+++ b/data/college-content-master.xlsx
@@ -2187,12 +2187,12 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Eligible - Auto Publish</t>
+          <t>Pushed - Awaiting Pages</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>

</xml_diff>